<commit_message>
Updated target_materials\Material_Types with Nitrocellulose HSP values.
</commit_message>
<xml_diff>
--- a/data/target_materials/Material_Types.xlsx
+++ b/data/target_materials/Material_Types.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sammo\Projects\HSP\data\target_materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{639A015F-5153-4361-B5BD-F76CC27DD4A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6732AFE7-C8D1-48DD-91CB-E7891C65D738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" tabRatio="668" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="82">
   <si>
     <t>δD</t>
   </si>
@@ -268,13 +268,16 @@
   </si>
   <si>
     <t>Material</t>
+  </si>
+  <si>
+    <t>Nitrocellulose (approximate)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -286,6 +289,13 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="6"/>
+      <color rgb="FF0A0A0A"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -323,7 +333,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -331,6 +341,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1340,15 +1351,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.46484375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4.73046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="3.73046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.73046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>79</v>
       </c>
@@ -1362,7 +1374,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>57</v>
       </c>
@@ -1376,7 +1388,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -1390,7 +1402,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>50</v>
       </c>
@@ -1404,7 +1416,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -1418,79 +1430,96 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6">
+        <v>15.8</v>
+      </c>
+      <c r="C6">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="D6">
+        <v>19.399999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
         <v>55</v>
       </c>
-      <c r="B6">
+      <c r="B7">
         <v>18</v>
       </c>
-      <c r="C6">
+      <c r="C7">
         <v>7</v>
       </c>
-      <c r="D6">
+      <c r="D7">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
         <v>49</v>
       </c>
-      <c r="B7">
+      <c r="B8">
         <v>17.5</v>
       </c>
-      <c r="C7">
+      <c r="C8">
         <v>8.5</v>
       </c>
-      <c r="D7">
+      <c r="D8">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
         <v>52</v>
       </c>
-      <c r="B8">
+      <c r="B9">
         <v>18</v>
       </c>
-      <c r="C8">
+      <c r="C9">
         <v>6</v>
       </c>
-      <c r="D8">
+      <c r="D9">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
         <v>56</v>
       </c>
-      <c r="B9">
+      <c r="B10">
         <v>17.5</v>
       </c>
-      <c r="C9">
+      <c r="C10">
         <v>5</v>
       </c>
-      <c r="D9">
+      <c r="D10">
         <v>8.5</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
         <v>54</v>
       </c>
-      <c r="B10">
+      <c r="B11">
         <v>17.2</v>
       </c>
-      <c r="C10">
+      <c r="C11">
         <v>4</v>
       </c>
-      <c r="D10">
+      <c r="D11">
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="H12" s="3"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D10">
-    <sortCondition ref="A1:A10"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D11">
+    <sortCondition ref="A1:A11"/>
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated again Nitrocellulose HSP values.
</commit_message>
<xml_diff>
--- a/data/target_materials/Material_Types.xlsx
+++ b/data/target_materials/Material_Types.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sammo\Projects\HSP\data\target_materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6732AFE7-C8D1-48DD-91CB-E7891C65D738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{490FA4D2-C89E-4569-987B-F655130C712F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" tabRatio="668" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1435,13 +1435,13 @@
         <v>81</v>
       </c>
       <c r="B6">
-        <v>15.8</v>
+        <v>16.2</v>
       </c>
       <c r="C6">
-        <v>8.8000000000000007</v>
+        <v>14.1</v>
       </c>
       <c r="D6">
-        <v>19.399999999999999</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">

</xml_diff>